<commit_message>
apos arrumar id de pack
</commit_message>
<xml_diff>
--- a/contas/alvesguilherme838@gmail.com/registros_pedidos.xlsx
+++ b/contas/alvesguilherme838@gmail.com/registros_pedidos.xlsx
@@ -4633,7 +4633,7 @@
         <v>424</v>
       </c>
       <c r="F131" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G131" t="s">
         <v>425</v>
@@ -4656,7 +4656,7 @@
         <v>424</v>
       </c>
       <c r="F132" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G132" t="s">
         <v>425</v>
@@ -4679,7 +4679,7 @@
         <v>424</v>
       </c>
       <c r="F133" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G133" t="s">
         <v>425</v>

</xml_diff>